<commit_message>
Fix Triangular editor values disappearing on sequential field edits
Replace syncInputsFromParams() with direct input state updates in blur
handlers to prevent race condition with useMultiParameterEditorState hook.
When setIsDirty(false) was called, the hook's effect would reset localParams
to original prop values before input sync completed, causing fields to clear.

Added regression test cases to Duration_Editor_Tests.xlsx for Triangular,
Uniform, and Normal distributions covering sequential field editing.

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_qa/Duration_Editor_Tests.xlsx
+++ b/_qa/Duration_Editor_Tests.xlsx
@@ -17,6 +17,153 @@
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="true"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+  <si>
+    <t>DUR-TRI-011</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>Sequential field editing (regression)</t>
+  </si>
+  <si>
+    <t>Triangular distribution selected</t>
+  </si>
+  <si>
+    <t>1. Enter 1 in Left, blur
+2. Enter 5 in Mode, blur
+3. Enter 10 in Right, blur</t>
+  </si>
+  <si>
+    <t>Left and Mode values remain visible after editing Right field</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Regression test for values disappearing bug</t>
+  </si>
+  <si>
+    <t>DUR-TRI-012</t>
+  </si>
+  <si>
+    <t>Values persist across all field changes</t>
+  </si>
+  <si>
+    <t>Triangular with left=1, mode=5, right=10</t>
+  </si>
+  <si>
+    <t>Edit each field in sequence: Left→Mode→Right, blurring after each</t>
+  </si>
+  <si>
+    <t>All three fields retain their values throughout editing</t>
+  </si>
+  <si>
+    <t>Tests direct input state updates in blur handlers</t>
+  </si>
+  <si>
+    <t>DUR-TRI-013</t>
+  </si>
+  <si>
+    <t>Cascade adjustment preserves other values</t>
+  </si>
+  <si>
+    <t>Set left=7 (triggering cascade), then edit right=15</t>
+  </si>
+  <si>
+    <t>After cascade: mode=8, right=9. After right edit: left=7, mode=8, right=15</t>
+  </si>
+  <si>
+    <t>Verifies cascade doesn't clear unrelated fields</t>
+  </si>
+  <si>
+    <t>DUR-UNI-009</t>
+  </si>
+  <si>
+    <t>Uniform distribution selected</t>
+  </si>
+  <si>
+    <t>1. Enter 5 in Low, blur
+2. Enter 15 in High, blur</t>
+  </si>
+  <si>
+    <t>Low value remains visible after editing High field</t>
+  </si>
+  <si>
+    <t>DUR-UNI-010</t>
+  </si>
+  <si>
+    <t>Values persist across field changes</t>
+  </si>
+  <si>
+    <t>Uniform with low=5, high=15</t>
+  </si>
+  <si>
+    <t>Edit Low to 3, blur. Edit High to 20, blur</t>
+  </si>
+  <si>
+    <t>Both fields retain values: Low=3, High=20</t>
+  </si>
+  <si>
+    <t>DUR-UNI-011</t>
+  </si>
+  <si>
+    <t>Cascade adjustment preserves other value</t>
+  </si>
+  <si>
+    <t>Set low=20 (triggering high cascade), then edit high=30</t>
+  </si>
+  <si>
+    <t>After cascade: high=21. After high edit: low=20, high=30</t>
+  </si>
+  <si>
+    <t>Verifies cascade doesn't clear the other field</t>
+  </si>
+  <si>
+    <t>DUR-NORM-009</t>
+  </si>
+  <si>
+    <t>Normal distribution selected</t>
+  </si>
+  <si>
+    <t>1. Enter 10 in Mean, blur
+2. Enter 2 in Std, blur</t>
+  </si>
+  <si>
+    <t>Mean value remains visible after editing Std field</t>
+  </si>
+  <si>
+    <t>DUR-NORM-010</t>
+  </si>
+  <si>
+    <t>Normal with mean=10, std=2</t>
+  </si>
+  <si>
+    <t>Edit Mean to 15, blur. Edit Std to 3, blur</t>
+  </si>
+  <si>
+    <t>Both fields retain values: Mean=15, Std=3</t>
+  </si>
+  <si>
+    <t>DUR-NORM-011</t>
+  </si>
+  <si>
+    <t>Edit both fields with decimals</t>
+  </si>
+  <si>
+    <t>Enter 7.5 in Mean, blur. Enter 1.25 in Std, blur</t>
+  </si>
+  <si>
+    <t>Both decimal values persist: Mean=7.5, Std=1.25</t>
+  </si>
+  <si>
+    <t>Tests decimal handling with sequential edits</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1176,7 +1323,7 @@
     <outlinePr summaryBelow="true" summaryRight="true"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1570,6 +1717,138 @@
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" t="s">
+        <v>6</v>
+      </c>
+      <c r="I10" t="s">
+        <v>6</v>
+      </c>
+      <c r="J10" t="s">
+        <v>6</v>
+      </c>
+      <c r="K10" t="s">
+        <v>6</v>
+      </c>
+      <c r="L10" t="s">
+        <v>6</v>
+      </c>
+      <c r="M10" t="s">
+        <v>7</v>
+      </c>
+      <c r="N10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" t="s">
+        <v>40</v>
+      </c>
+      <c r="G11" t="s">
+        <v>6</v>
+      </c>
+      <c r="H11" t="s">
+        <v>6</v>
+      </c>
+      <c r="I11" t="s">
+        <v>6</v>
+      </c>
+      <c r="J11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K11" t="s">
+        <v>6</v>
+      </c>
+      <c r="L11" t="s">
+        <v>6</v>
+      </c>
+      <c r="M11" t="s">
+        <v>13</v>
+      </c>
+      <c r="N11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" t="s">
+        <v>43</v>
+      </c>
+      <c r="F12" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I12" t="s">
+        <v>6</v>
+      </c>
+      <c r="J12" t="s">
+        <v>6</v>
+      </c>
+      <c r="K12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L12" t="s">
+        <v>6</v>
+      </c>
+      <c r="M12" t="s">
+        <v>45</v>
+      </c>
+      <c r="N12" t="s">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1582,7 +1861,7 @@
     <outlinePr summaryBelow="true" summaryRight="true"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1976,6 +2255,138 @@
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" t="s">
+        <v>6</v>
+      </c>
+      <c r="I10" t="s">
+        <v>6</v>
+      </c>
+      <c r="J10" t="s">
+        <v>6</v>
+      </c>
+      <c r="K10" t="s">
+        <v>6</v>
+      </c>
+      <c r="L10" t="s">
+        <v>6</v>
+      </c>
+      <c r="M10" t="s">
+        <v>7</v>
+      </c>
+      <c r="N10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" t="s">
+        <v>6</v>
+      </c>
+      <c r="H11" t="s">
+        <v>6</v>
+      </c>
+      <c r="I11" t="s">
+        <v>6</v>
+      </c>
+      <c r="J11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K11" t="s">
+        <v>6</v>
+      </c>
+      <c r="L11" t="s">
+        <v>6</v>
+      </c>
+      <c r="M11" t="s">
+        <v>13</v>
+      </c>
+      <c r="N11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I12" t="s">
+        <v>6</v>
+      </c>
+      <c r="J12" t="s">
+        <v>6</v>
+      </c>
+      <c r="K12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L12" t="s">
+        <v>6</v>
+      </c>
+      <c r="M12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N12" t="s">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1988,7 +2399,7 @@
     <outlinePr summaryBelow="true" summaryRight="true"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2462,6 +2873,138 @@
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" t="s">
+        <v>4</v>
+      </c>
+      <c r="F12" t="s">
+        <v>5</v>
+      </c>
+      <c r="G12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I12" t="s">
+        <v>6</v>
+      </c>
+      <c r="J12" t="s">
+        <v>6</v>
+      </c>
+      <c r="K12" t="s">
+        <v>6</v>
+      </c>
+      <c r="L12" t="s">
+        <v>6</v>
+      </c>
+      <c r="M12" t="s">
+        <v>7</v>
+      </c>
+      <c r="N12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" t="s">
+        <v>6</v>
+      </c>
+      <c r="H13" t="s">
+        <v>6</v>
+      </c>
+      <c r="I13" t="s">
+        <v>6</v>
+      </c>
+      <c r="J13" t="s">
+        <v>6</v>
+      </c>
+      <c r="K13" t="s">
+        <v>6</v>
+      </c>
+      <c r="L13" t="s">
+        <v>6</v>
+      </c>
+      <c r="M13" t="s">
+        <v>13</v>
+      </c>
+      <c r="N13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" t="s">
+        <v>6</v>
+      </c>
+      <c r="H14" t="s">
+        <v>6</v>
+      </c>
+      <c r="I14" t="s">
+        <v>6</v>
+      </c>
+      <c r="J14" t="s">
+        <v>6</v>
+      </c>
+      <c r="K14" t="s">
+        <v>6</v>
+      </c>
+      <c r="L14" t="s">
+        <v>6</v>
+      </c>
+      <c r="M14" t="s">
+        <v>18</v>
+      </c>
+      <c r="N14" t="s">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>